<commit_message>
feat: add batch mode for expand and rank graph.
- revise expand_and_rank_graph, use function parameters instead of hard code paths.
- add batch_expand_and_rank_graph.py, run multiple projects at once.
- change some SOURCE_DIR, not use that in lowcode_public.
</commit_message>
<xml_diff>
--- a/src/generation/dev_eval/project_to_run/0311_5projects.xlsx
+++ b/src/generation/dev_eval/project_to_run/0311_5projects.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xianlin/Desktop/25-26/26-03/批量跑项目/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AC32048F-1313-634B-8B77-43F738CE7ABB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEACD014-E2D9-9144-82A1-BFA6FD4C6722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15180" yWindow="9400" windowWidth="27440" windowHeight="16440" xr2:uid="{011B4B81-92DE-A948-A522-FCF23BAD9B78}"/>
+    <workbookView xWindow="12460" yWindow="5160" windowWidth="27440" windowHeight="16440" xr2:uid="{011B4B81-92DE-A948-A522-FCF23BAD9B78}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -61,24 +61,19 @@
     <t>mingus</t>
   </si>
   <si>
-    <t>/data/lowcode_public/DevEval/Source_Code/System/mrjob</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>/data/lowcode_public/DevEval/Source_Code/Internet/boto</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>/data/lowcode_public/DevEval/Source_Code/Database/alembic</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>/data/lowcode_public/DevEval/Source_Code/Security/diffprivlib</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>/data/lowcode_public/DevEval/Source_Code/Multimedia/mingus</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+    <t>/data/zxl/Search2026/Datasets/Source_Code/System/mrjob</t>
+  </si>
+  <si>
+    <t>/data/zxl/Search2026/Datasets/Source_Code/Internet/boto</t>
+  </si>
+  <si>
+    <t>/data/zxl/Search2026/Datasets/Source_Code/Database/alembic</t>
+  </si>
+  <si>
+    <t>/data/zxl/Search2026/Datasets/Source_Code/Security/diffprivlib</t>
+  </si>
+  <si>
+    <t>/data/zxl/Search2026/Datasets/Source_Code/Multimedia/mingus</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
feat: add code len calculation.
</commit_message>
<xml_diff>
--- a/src/generation/dev_eval/project_to_run/0311_5projects.xlsx
+++ b/src/generation/dev_eval/project_to_run/0311_5projects.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xianlin/Desktop/25-26/26-03/批量跑项目/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEACD014-E2D9-9144-82A1-BFA6FD4C6722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD846506-5D63-5945-86BC-D27CF906385A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12460" yWindow="5160" windowWidth="27440" windowHeight="16440" xr2:uid="{011B4B81-92DE-A948-A522-FCF23BAD9B78}"/>
+    <workbookView xWindow="13520" yWindow="8160" windowWidth="27440" windowHeight="16440" xr2:uid="{011B4B81-92DE-A948-A522-FCF23BAD9B78}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -61,19 +61,24 @@
     <t>mingus</t>
   </si>
   <si>
-    <t>/data/zxl/Search2026/Datasets/Source_Code/System/mrjob</t>
-  </si>
-  <si>
-    <t>/data/zxl/Search2026/Datasets/Source_Code/Internet/boto</t>
-  </si>
-  <si>
-    <t>/data/zxl/Search2026/Datasets/Source_Code/Database/alembic</t>
-  </si>
-  <si>
-    <t>/data/zxl/Search2026/Datasets/Source_Code/Security/diffprivlib</t>
-  </si>
-  <si>
-    <t>/data/zxl/Search2026/Datasets/Source_Code/Multimedia/mingus</t>
+    <t>/data/zxl/Search2026/Datasets/Source_Code/System/mrjob/mrjob</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/data/zxl/Search2026/Datasets/Source_Code/Internet/boto/boto</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/data/zxl/Search2026/Datasets/Source_Code/Database/alembic/alembic</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/data/zxl/Search2026/Datasets/Source_Code/Security/diffprivlib/diffprivlib</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/data/zxl/Search2026/Datasets/Source_Code/Multimedia/mingus/mingus</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>

</xml_diff>